<commit_message>
chore: deployment update 2026-03-05 19:04:09
</commit_message>
<xml_diff>
--- a/final_grades_filled.xlsx
+++ b/final_grades_filled.xlsx
@@ -34,7 +34,7 @@
     <t>O210008</t>
   </si>
   <si>
-    <t>SreeCharan Niggs</t>
+    <t>SreeCharan Daamu</t>
   </si>
   <si>
     <t>CSE-E2-SEM-1-01</t>
@@ -46,39 +46,42 @@
     <t>E2-SEM-1</t>
   </si>
   <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>CSE-E2-SEM-1-02</t>
+  </si>
+  <si>
+    <t>Digital Logic Design</t>
+  </si>
+  <si>
+    <t>EX</t>
+  </si>
+  <si>
+    <t>CSE-E2-SEM-1-03</t>
+  </si>
+  <si>
+    <t>Design &amp; Analysis of Algorithms</t>
+  </si>
+  <si>
+    <t>CSE-E2-SEM-1-04</t>
+  </si>
+  <si>
+    <t>Database Management Systems</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>CSE-E2-SEM-1-05</t>
+  </si>
+  <si>
+    <t>Formal Languages &amp; Automata Theory</t>
+  </si>
+  <si>
     <t>A</t>
   </si>
   <si>
-    <t>CSE-E2-SEM-1-02</t>
-  </si>
-  <si>
-    <t>Digital Logic Design</t>
-  </si>
-  <si>
-    <t>CSE-E2-SEM-1-03</t>
-  </si>
-  <si>
-    <t>Design &amp; Analysis of Algorithms</t>
-  </si>
-  <si>
-    <t>CSE-E2-SEM-1-04</t>
-  </si>
-  <si>
-    <t>Database Management Systems</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>CSE-E2-SEM-1-05</t>
-  </si>
-  <si>
-    <t>Formal Languages &amp; Automata Theory</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>CSE-E2-SEM-1-06</t>
   </si>
   <si>
@@ -89,9 +92,6 @@
   </si>
   <si>
     <t>Digital Logic Design Lab</t>
-  </si>
-  <si>
-    <t>E</t>
   </si>
   <si>
     <t>CSE-E2-SEM-1-08</t>
@@ -555,7 +555,7 @@
         <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -566,10 +566,10 @@
         <v>7</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>10</v>
@@ -586,16 +586,16 @@
         <v>7</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -606,16 +606,16 @@
         <v>7</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -626,16 +626,16 @@
         <v>7</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -646,16 +646,16 @@
         <v>7</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -675,7 +675,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: deployment update 2026-03-05 19:09:51
</commit_message>
<xml_diff>
--- a/final_grades_filled.xlsx
+++ b/final_grades_filled.xlsx
@@ -46,42 +46,39 @@
     <t>E2-SEM-1</t>
   </si>
   <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>CSE-E2-SEM-1-02</t>
+  </si>
+  <si>
+    <t>Digital Logic Design</t>
+  </si>
+  <si>
+    <t>EX</t>
+  </si>
+  <si>
+    <t>CSE-E2-SEM-1-03</t>
+  </si>
+  <si>
+    <t>Design &amp; Analysis of Algorithms</t>
+  </si>
+  <si>
     <t>B</t>
   </si>
   <si>
-    <t>CSE-E2-SEM-1-02</t>
-  </si>
-  <si>
-    <t>Digital Logic Design</t>
-  </si>
-  <si>
-    <t>EX</t>
-  </si>
-  <si>
-    <t>CSE-E2-SEM-1-03</t>
-  </si>
-  <si>
-    <t>Design &amp; Analysis of Algorithms</t>
-  </si>
-  <si>
     <t>CSE-E2-SEM-1-04</t>
   </si>
   <si>
     <t>Database Management Systems</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>CSE-E2-SEM-1-05</t>
   </si>
   <si>
     <t>Formal Languages &amp; Automata Theory</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>CSE-E2-SEM-1-06</t>
   </si>
   <si>
@@ -92,6 +89,9 @@
   </si>
   <si>
     <t>Digital Logic Design Lab</t>
+  </si>
+  <si>
+    <t>D</t>
   </si>
   <si>
     <t>CSE-E2-SEM-1-08</t>
@@ -575,7 +575,7 @@
         <v>10</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -586,16 +586,16 @@
         <v>7</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -615,7 +615,7 @@
         <v>10</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -626,16 +626,16 @@
         <v>7</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -646,16 +646,16 @@
         <v>7</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -675,7 +675,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>